<commit_message>
Update manuscript code and documentation
</commit_message>
<xml_diff>
--- a/forewing_data/refs.xlsx
+++ b/forewing_data/refs.xlsx
@@ -1,8 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\16240\Desktop\air\dimensionless\New\github_open\forewing_data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView windowWidth="24750" windowHeight="10480"/>
   </bookViews>
@@ -29,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Reference</t>
   </si>
@@ -49,13 +54,14 @@
     <t>[2]</t>
   </si>
   <si>
-    <t>Weibin Gu. Internet dataset 2</t>
+    <t>Weibin Gu. Internet dataset//W. Gu, C. Feng, L. Liu, C. Yang, X. Jiao, Y. Ding, X. Shi,
+C. Gao, A. Rizzo, and G. Zhou, “A 26-Gram Tailless
+Butterfly-Inspired Flapping-Wing Robot with Onboard
+Attitude Control”, arXiv preprint arXiv:2602.06811v3
+(2026)</t>
   </si>
   <si>
     <t>[3]</t>
-  </si>
-  <si>
-    <t>Weibin Gu. Internet dataset 1</t>
   </si>
   <si>
     <t>[4]</t>
@@ -733,7 +739,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -745,9 +751,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1094,10 +1097,10 @@
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="2">
         <v>9</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <f>SUM(C:C)</f>
         <v>383</v>
       </c>
@@ -1109,58 +1112,58 @@
       <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="2">
         <v>10</v>
       </c>
-      <c r="D3" s="4"/>
+      <c r="D3" s="2"/>
     </row>
     <row r="4" ht="22.5" customHeight="1" spans="1:4">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2">
         <v>9</v>
       </c>
-      <c r="D4" s="4"/>
+      <c r="D4" s="2"/>
     </row>
     <row r="5" ht="88.5" customHeight="1" spans="1:4">
       <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4">
+      <c r="C5" s="2">
         <v>1</v>
       </c>
-      <c r="D5" s="4"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6" ht="39" customHeight="1" spans="1:4">
       <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="4">
+      <c r="C6" s="2">
         <v>66</v>
       </c>
-      <c r="D6" s="4"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" ht="22.5" customHeight="1" spans="1:4">
       <c r="A7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="4">
+      <c r="C7" s="2">
         <v>288</v>
       </c>
-      <c r="D7" s="4"/>
+      <c r="D7" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>